<commit_message>
THÁNG 10: dùng công thức SUM đơn giản cho cột TỔNG ngày
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0157QgvJhh2coHDAY77Q3zK5
</commit_message>
<xml_diff>
--- a/SoTheoDoiThuChi_T10_2026.xlsx
+++ b/SoTheoDoiThuChi_T10_2026.xlsx
@@ -7481,11 +7481,11 @@
       <c r="E5" s="31"/>
       <c r="F5" s="31"/>
       <c r="G5" s="38" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A5,$B$5:$B$504,B5)+SUMIFS($E$5:$E$504,$A$5:$A$504,A5,$B$5:$B$504,B5)-SUMIFS($F$5:$F$504,$A$5:$A$504,A5,$B$5:$B$504,B5)</f>
+        <f aca="false">SUM(D5:D13)+SUM(E5:E13)-SUM(F5:F13)</f>
         <v>34142</v>
       </c>
       <c r="H5" s="38" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A5,$B$5:$B$504,B5)</f>
+        <f aca="false">SUM(F5:F13)</f>
         <v>408</v>
       </c>
       <c r="I5" s="39" t="s">
@@ -7695,11 +7695,11 @@
         <v>206</v>
       </c>
       <c r="G14" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A14,$B$5:$B$504,B14)+SUMIFS($E$5:$E$504,$A$5:$A$504,A14,$B$5:$B$504,B14)-SUMIFS($F$5:$F$504,$A$5:$A$504,A14,$B$5:$B$504,B14)</f>
+        <f aca="false">SUM(D14:D19)+SUM(E14:E19)-SUM(F14:F19)</f>
         <v>18689</v>
       </c>
       <c r="H14" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A14,$B$5:$B$504,B14)</f>
+        <f aca="false">SUM(F14:F19)</f>
         <v>1161</v>
       </c>
       <c r="I14" s="44" t="s">
@@ -7841,11 +7841,11 @@
       </c>
       <c r="F20" s="42"/>
       <c r="G20" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A20,$B$5:$B$504,B20)+SUMIFS($E$5:$E$504,$A$5:$A$504,A20,$B$5:$B$504,B20)-SUMIFS($F$5:$F$504,$A$5:$A$504,A20,$B$5:$B$504,B20)</f>
+        <f aca="false">SUM(D20:D21)+SUM(E20:E21)-SUM(F20:F21)</f>
         <v>9250</v>
       </c>
       <c r="H20" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A20,$B$5:$B$504,B20)</f>
+        <f aca="false">SUM(F20:F21)</f>
         <v>0</v>
       </c>
       <c r="I20" s="44" t="s">
@@ -7891,11 +7891,11 @@
       </c>
       <c r="F22" s="42"/>
       <c r="G22" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A22,$B$5:$B$504,B22)+SUMIFS($E$5:$E$504,$A$5:$A$504,A22,$B$5:$B$504,B22)-SUMIFS($F$5:$F$504,$A$5:$A$504,A22,$B$5:$B$504,B22)</f>
+        <f aca="false">D22+E22-F22</f>
         <v>10000</v>
       </c>
       <c r="H22" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A22,$B$5:$B$504,B22)</f>
+        <f aca="false">F22</f>
         <v>0</v>
       </c>
       <c r="I22" s="44" t="s">
@@ -7921,11 +7921,11 @@
         <v>700</v>
       </c>
       <c r="G23" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A23,$B$5:$B$504,B23)+SUMIFS($E$5:$E$504,$A$5:$A$504,A23,$B$5:$B$504,B23)-SUMIFS($F$5:$F$504,$A$5:$A$504,A23,$B$5:$B$504,B23)</f>
+        <f aca="false">D23+E23-F23</f>
         <v>-650</v>
       </c>
       <c r="H23" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A23,$B$5:$B$504,B23)</f>
+        <f aca="false">F23</f>
         <v>700</v>
       </c>
       <c r="I23" s="44" t="s">
@@ -7953,11 +7953,11 @@
         <v>100</v>
       </c>
       <c r="G24" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A24,$B$5:$B$504,B24)+SUMIFS($E$5:$E$504,$A$5:$A$504,A24,$B$5:$B$504,B24)-SUMIFS($F$5:$F$504,$A$5:$A$504,A24,$B$5:$B$504,B24)</f>
+        <f aca="false">SUM(D24:D28)+SUM(E24:E28)-SUM(F24:F28)</f>
         <v>8000</v>
       </c>
       <c r="H24" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A24,$B$5:$B$504,B24)</f>
+        <f aca="false">SUM(F24:F28)</f>
         <v>200</v>
       </c>
       <c r="I24" s="44" t="s">
@@ -8073,11 +8073,11 @@
       <c r="E29" s="42"/>
       <c r="F29" s="42"/>
       <c r="G29" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A29,$B$5:$B$504,B29)+SUMIFS($E$5:$E$504,$A$5:$A$504,A29,$B$5:$B$504,B29)-SUMIFS($F$5:$F$504,$A$5:$A$504,A29,$B$5:$B$504,B29)</f>
+        <f aca="false">SUM(D29:D30)+SUM(E29:E30)-SUM(F29:F30)</f>
         <v>150</v>
       </c>
       <c r="H29" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A29,$B$5:$B$504,B29)</f>
+        <f aca="false">SUM(F29:F30)</f>
         <v>0</v>
       </c>
       <c r="I29" s="44" t="s">
@@ -8123,11 +8123,11 @@
       <c r="E31" s="42"/>
       <c r="F31" s="42"/>
       <c r="G31" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A31,$B$5:$B$504,B31)+SUMIFS($E$5:$E$504,$A$5:$A$504,A31,$B$5:$B$504,B31)-SUMIFS($F$5:$F$504,$A$5:$A$504,A31,$B$5:$B$504,B31)</f>
+        <f aca="false">SUM(D31:D37)+SUM(E31:E37)-SUM(F31:F37)</f>
         <v>16810</v>
       </c>
       <c r="H31" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A31,$B$5:$B$504,B31)</f>
+        <f aca="false">SUM(F31:F37)</f>
         <v>1120</v>
       </c>
       <c r="I31" s="44" t="s">
@@ -8285,11 +8285,11 @@
       <c r="E38" s="42"/>
       <c r="F38" s="42"/>
       <c r="G38" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A38,$B$5:$B$504,B38)+SUMIFS($E$5:$E$504,$A$5:$A$504,A38,$B$5:$B$504,B38)-SUMIFS($F$5:$F$504,$A$5:$A$504,A38,$B$5:$B$504,B38)</f>
+        <f aca="false">SUM(D38:D46)+SUM(E38:E46)-SUM(F38:F46)</f>
         <v>25590</v>
       </c>
       <c r="H38" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A38,$B$5:$B$504,B38)</f>
+        <f aca="false">SUM(F38:F46)</f>
         <v>0</v>
       </c>
       <c r="I38" s="44" t="s">
@@ -8489,11 +8489,11 @@
       <c r="E47" s="42"/>
       <c r="F47" s="42"/>
       <c r="G47" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A47,$B$5:$B$504,B47)+SUMIFS($E$5:$E$504,$A$5:$A$504,A47,$B$5:$B$504,B47)-SUMIFS($F$5:$F$504,$A$5:$A$504,A47,$B$5:$B$504,B47)</f>
+        <f aca="false">SUM(D47:D49)+SUM(E47:E49)-SUM(F47:F49)</f>
         <v>5550</v>
       </c>
       <c r="H47" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A47,$B$5:$B$504,B47)</f>
+        <f aca="false">SUM(F47:F49)</f>
         <v>0</v>
       </c>
       <c r="I47" s="44" t="s">
@@ -8563,11 +8563,11 @@
       <c r="E50" s="42"/>
       <c r="F50" s="42"/>
       <c r="G50" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A50,$B$5:$B$504,B50)+SUMIFS($E$5:$E$504,$A$5:$A$504,A50,$B$5:$B$504,B50)-SUMIFS($F$5:$F$504,$A$5:$A$504,A50,$B$5:$B$504,B50)</f>
+        <f aca="false">SUM(D50:D51)+SUM(E50:E51)-SUM(F50:F51)</f>
         <v>9</v>
       </c>
       <c r="H50" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A50,$B$5:$B$504,B50)</f>
+        <f aca="false">SUM(F50:F51)</f>
         <v>251</v>
       </c>
       <c r="I50" s="44" t="s">
@@ -8615,11 +8615,11 @@
       <c r="E52" s="42"/>
       <c r="F52" s="42"/>
       <c r="G52" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A52,$B$5:$B$504,B52)+SUMIFS($E$5:$E$504,$A$5:$A$504,A52,$B$5:$B$504,B52)-SUMIFS($F$5:$F$504,$A$5:$A$504,A52,$B$5:$B$504,B52)</f>
+        <f aca="false">D52+E52-F52</f>
         <v>50</v>
       </c>
       <c r="H52" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A52,$B$5:$B$504,B52)</f>
+        <f aca="false">F52</f>
         <v>0</v>
       </c>
       <c r="I52" s="44" t="s">
@@ -8647,11 +8647,11 @@
         <v>500</v>
       </c>
       <c r="G53" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A53,$B$5:$B$504,B53)+SUMIFS($E$5:$E$504,$A$5:$A$504,A53,$B$5:$B$504,B53)-SUMIFS($F$5:$F$504,$A$5:$A$504,A53,$B$5:$B$504,B53)</f>
+        <f aca="false">D53+E53-F53</f>
         <v>11900</v>
       </c>
       <c r="H53" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A53,$B$5:$B$504,B53)</f>
+        <f aca="false">F53</f>
         <v>500</v>
       </c>
       <c r="I53" s="44" t="s">
@@ -8675,11 +8675,11 @@
       <c r="E54" s="42"/>
       <c r="F54" s="42"/>
       <c r="G54" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A54,$B$5:$B$504,B54)+SUMIFS($E$5:$E$504,$A$5:$A$504,A54,$B$5:$B$504,B54)-SUMIFS($F$5:$F$504,$A$5:$A$504,A54,$B$5:$B$504,B54)</f>
+        <f aca="false">D54+E54-F54</f>
         <v>100</v>
       </c>
       <c r="H54" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A54,$B$5:$B$504,B54)</f>
+        <f aca="false">F54</f>
         <v>0</v>
       </c>
       <c r="I54" s="44" t="s">
@@ -8703,11 +8703,11 @@
       </c>
       <c r="F55" s="49"/>
       <c r="G55" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A55,$B$5:$B$504,B55)+SUMIFS($E$5:$E$504,$A$5:$A$504,A55,$B$5:$B$504,B55)-SUMIFS($F$5:$F$504,$A$5:$A$504,A55,$B$5:$B$504,B55)</f>
+        <f aca="false">D55+E55-F55</f>
         <v>4600</v>
       </c>
       <c r="H55" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A55,$B$5:$B$504,B55)</f>
+        <f aca="false">F55</f>
         <v>0</v>
       </c>
       <c r="I55" s="50" t="s">
@@ -8733,11 +8733,11 @@
       <c r="E56" s="42"/>
       <c r="F56" s="42"/>
       <c r="G56" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A56,$B$5:$B$504,B56)+SUMIFS($E$5:$E$504,$A$5:$A$504,A56,$B$5:$B$504,B56)-SUMIFS($F$5:$F$504,$A$5:$A$504,A56,$B$5:$B$504,B56)</f>
+        <f aca="false">SUM(D56:D58)+SUM(E56:E58)-SUM(F56:F58)</f>
         <v>250</v>
       </c>
       <c r="H56" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A56,$B$5:$B$504,B56)</f>
+        <f aca="false">SUM(F56:F58)</f>
         <v>500</v>
       </c>
       <c r="I56" s="44" t="s">
@@ -8859,11 +8859,11 @@
       <c r="E61" s="42"/>
       <c r="F61" s="42"/>
       <c r="G61" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A61,$B$5:$B$504,B61)+SUMIFS($E$5:$E$504,$A$5:$A$504,A61,$B$5:$B$504,B61)-SUMIFS($F$5:$F$504,$A$5:$A$504,A61,$B$5:$B$504,B61)</f>
+        <f aca="false">D61+E61-F61</f>
         <v>1000</v>
       </c>
       <c r="H61" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A61,$B$5:$B$504,B61)</f>
+        <f aca="false">F61</f>
         <v>0</v>
       </c>
       <c r="I61" s="44" t="s">
@@ -8887,11 +8887,11 @@
       <c r="E62" s="42"/>
       <c r="F62" s="42"/>
       <c r="G62" s="43" t="n">
-        <f aca="false">SUMIFS($D$5:$D$504,$A$5:$A$504,A62,$B$5:$B$504,B62)+SUMIFS($E$5:$E$504,$A$5:$A$504,A62,$B$5:$B$504,B62)-SUMIFS($F$5:$F$504,$A$5:$A$504,A62,$B$5:$B$504,B62)</f>
+        <f aca="false">D62+E62-F62</f>
         <v>2500</v>
       </c>
       <c r="H62" s="43" t="n">
-        <f aca="false">SUMIFS($F$5:$F$504,$A$5:$A$504,A62,$B$5:$B$504,B62)</f>
+        <f aca="false">F62</f>
         <v>0</v>
       </c>
       <c r="I62" s="44" t="s">

</xml_diff>